<commit_message>
fix: exclude gadget balance from operator markers
</commit_message>
<xml_diff>
--- a/docs/主武器射速榜.xlsx
+++ b/docs/主武器射速榜.xlsx
@@ -10215,7 +10215,7 @@
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -10249,7 +10249,7 @@
       <c r="V3" s="5" t="n"/>
       <c r="W3" s="8" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="7" t="inlineStr">
@@ -10514,7 +10514,7 @@
       <c r="AB7" s="5" t="n"/>
       <c r="AC7" s="9" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AD7" s="7" t="inlineStr">
@@ -10745,7 +10745,7 @@
       <c r="V11" s="5" t="n"/>
       <c r="W11" s="17" t="inlineStr">
         <is>
-          <t>F+</t>
+          <t>F</t>
         </is>
       </c>
       <c r="X11" s="7" t="inlineStr">
@@ -10964,7 +10964,7 @@
       <c r="J15" s="5" t="n"/>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -11212,7 +11212,7 @@
       <c r="J19" s="5" t="n"/>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
@@ -11471,7 +11471,7 @@
       <c r="V23" s="5" t="n"/>
       <c r="W23" s="8" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X23" s="7" t="inlineStr">
@@ -11702,7 +11702,7 @@
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="10" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>C</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr">
@@ -11719,7 +11719,7 @@
       <c r="V27" s="5" t="n"/>
       <c r="W27" s="17" t="inlineStr">
         <is>
-          <t>F+</t>
+          <t>F</t>
         </is>
       </c>
       <c r="X27" s="7" t="inlineStr">
@@ -11910,7 +11910,7 @@
       <c r="J31" s="5" t="n"/>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L31" s="7" t="inlineStr">
@@ -11944,7 +11944,7 @@
       <c r="V31" s="5" t="n"/>
       <c r="W31" s="21" t="inlineStr">
         <is>
-          <t>D+</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X31" s="7" t="inlineStr">

</xml_diff>